<commit_message>
HST GO 18055 Processing Update
Did significant work updating processing. Now can plot empirically corrected patches of HST data and compare to SCT data.
</commit_message>
<xml_diff>
--- a/Catalog/Catalog-static.xlsx
+++ b/Catalog/Catalog-static.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Astronomy\Projects\SAS 2021 Ammonia\Jupiter_NH3_Analysis_P3\Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A7DC70-4E54-446D-A224-0DF26005EE83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E58B082-47C5-4462-AB28-2DEDC0A213F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Catalog-static" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5874" uniqueCount="2451">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5887" uniqueCount="2457">
   <si>
     <t>ObsID</t>
   </si>
@@ -7419,12 +7419,6 @@
     <t>Took lots more, but they were clouded. Some of these have low SNR due to clouds</t>
   </si>
   <si>
-    <t>Very clear when I started very poor later, possibly the best seeing this apparition</t>
-  </si>
-  <si>
-    <t>Very clear and pretty good seeing</t>
-  </si>
-  <si>
     <t>Very clear initially, pretty good seeing. Got clouded out about 3:45am LT</t>
   </si>
   <si>
@@ -7486,9 +7480,6 @@
     <t>Very clear. Good seeing once Jupiter was high enough above the horizon</t>
   </si>
   <si>
-    <t>Very clear, very good seeing (expected from GFS). Extraordinary seeing at 11:35pm LT</t>
-  </si>
-  <si>
     <t>Very clear, very good seeing (not quite as good as the prior night)</t>
   </si>
   <si>
@@ -7496,6 +7487,69 @@
   </si>
   <si>
     <t>Very clear, very good seeing. Had power interrupt lost 20 mins, then later found mount clock was wrong and lost about 65 mins around flip</t>
+  </si>
+  <si>
+    <t>Some haze to start, then clearing, then clouds again. Seeing was good</t>
+  </si>
+  <si>
+    <t>Some haze to start, then very clear. Seeing was very good</t>
+  </si>
+  <si>
+    <t>Very good seeing. Very transparent</t>
+  </si>
+  <si>
+    <t>Ready for Nav</t>
+  </si>
+  <si>
+    <r>
+      <t>Very clear when I started very poor later,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> possibly the best seeing this apparition</t>
+    </r>
+  </si>
+  <si>
+    <t>Very clear and pretty good (maybe fair to poor) seeing</t>
+  </si>
+  <si>
+    <r>
+      <t>Very clear,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> very good seeing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (expected from GFS). Extraordinary seeing at 11:35pm LT</t>
+    </r>
+  </si>
+  <si>
+    <t>Good seeing. Clear, then clouds came in</t>
+  </si>
+  <si>
+    <t>Very good seeing. Very transparent. Extraordinary seeing in the middle of the night. Maybe 24 of 27 are very good quality.</t>
   </si>
 </sst>
 </file>
@@ -40313,10 +40367,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FB822E-4FB0-4362-8846-871BD8F7A1EF}">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E617"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.81640625" customWidth="1"/>
     <col min="4" max="4" width="12.7265625" customWidth="1"/>
     <col min="5" max="5" width="47.54296875" customWidth="1"/>
@@ -40327,8 +40382,8 @@
         <v>685</v>
       </c>
       <c r="B1" s="18">
-        <f>SUM(B2:B101)</f>
-        <v>986</v>
+        <f>SUM(B2:B151)</f>
+        <v>1135</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>696</v>
@@ -41189,7 +41244,7 @@
         <v>20</v>
       </c>
       <c r="E58" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
@@ -41200,7 +41255,7 @@
         <v>13</v>
       </c>
       <c r="E59" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
@@ -41258,7 +41313,7 @@
         <v>695</v>
       </c>
       <c r="E64" s="18" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
@@ -41272,7 +41327,7 @@
         <v>695</v>
       </c>
       <c r="E65" t="s">
-        <v>2444</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
@@ -41371,9 +41426,11 @@
         <f>198/22</f>
         <v>9</v>
       </c>
-      <c r="D74" s="51"/>
+      <c r="D74" s="58" t="s">
+        <v>2451</v>
+      </c>
       <c r="E74" s="18" t="s">
-        <v>2438</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
@@ -41383,9 +41440,11 @@
       <c r="B75">
         <v>27</v>
       </c>
-      <c r="D75" s="51"/>
+      <c r="D75" s="58" t="s">
+        <v>2451</v>
+      </c>
       <c r="E75" t="s">
-        <v>2439</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
@@ -41395,9 +41454,14 @@
       <c r="B76">
         <v>19</v>
       </c>
-      <c r="D76" s="58"/>
+      <c r="C76" t="s">
+        <v>687</v>
+      </c>
+      <c r="D76" s="58" t="s">
+        <v>2451</v>
+      </c>
       <c r="E76" t="s">
-        <v>2440</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
@@ -41407,9 +41471,14 @@
       <c r="B77">
         <v>28</v>
       </c>
-      <c r="D77" s="58"/>
+      <c r="C77" t="s">
+        <v>687</v>
+      </c>
+      <c r="D77" s="58" t="s">
+        <v>2451</v>
+      </c>
       <c r="E77" t="s">
-        <v>2445</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
@@ -41419,9 +41488,9 @@
       <c r="B78">
         <v>26</v>
       </c>
-      <c r="D78" s="51"/>
+      <c r="D78" s="58"/>
       <c r="E78" t="s">
-        <v>2446</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
@@ -41431,9 +41500,11 @@
       <c r="B79">
         <v>27</v>
       </c>
-      <c r="D79" s="51"/>
+      <c r="D79" s="58" t="s">
+        <v>2451</v>
+      </c>
       <c r="E79" t="s">
-        <v>2447</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
@@ -41445,7 +41516,7 @@
       </c>
       <c r="D80" s="51"/>
       <c r="E80" t="s">
-        <v>2448</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
@@ -41456,7 +41527,7 @@
         <v>26</v>
       </c>
       <c r="E81" t="s">
-        <v>2449</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
@@ -41467,15 +41538,1661 @@
         <v>26</v>
       </c>
       <c r="E82" t="s">
+        <v>2447</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A83" s="30">
+        <v>46034</v>
+      </c>
+      <c r="B83">
+        <v>27</v>
+      </c>
+      <c r="E83" t="s">
+        <v>2449</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A84" s="30">
+        <v>45670</v>
+      </c>
+      <c r="B84">
+        <v>23</v>
+      </c>
+      <c r="E84" t="s">
+        <v>2448</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A85" s="30">
+        <v>46037</v>
+      </c>
+      <c r="B85">
+        <v>28</v>
+      </c>
+      <c r="E85" t="s">
         <v>2450</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A83" s="30"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A84" s="30"/>
-      <c r="B84" s="30"/>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A86" s="30">
+        <v>46040</v>
+      </c>
+      <c r="B86">
+        <v>26</v>
+      </c>
+      <c r="E86" t="s">
+        <v>2450</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A87" s="30">
+        <v>46042</v>
+      </c>
+      <c r="B87">
+        <v>18</v>
+      </c>
+      <c r="E87" t="s">
+        <v>2455</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A88" s="30">
+        <v>46050</v>
+      </c>
+      <c r="B88">
+        <v>27</v>
+      </c>
+      <c r="E88" t="s">
+        <v>2456</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A89" s="30"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A90" s="30"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" s="30"/>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" s="30"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A93" s="30"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" s="30"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" s="30"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" s="30"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" s="30"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" s="30"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" s="30"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" s="30"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" s="30"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" s="30"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" s="30"/>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" s="30"/>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" s="30"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" s="30"/>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" s="30"/>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A108" s="30"/>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A109" s="30"/>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A110" s="30"/>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A111" s="30"/>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A112" s="30"/>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113" s="30"/>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A114" s="30"/>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A115" s="30"/>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A116" s="30"/>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A117" s="30"/>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A118" s="30"/>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A119" s="30"/>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A120" s="30"/>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A121" s="30"/>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A122" s="30"/>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A123" s="30"/>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A124" s="30"/>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A125" s="30"/>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A126" s="30"/>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A127" s="30"/>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A128" s="30"/>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A129" s="30"/>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A130" s="30"/>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A131" s="30"/>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A132" s="30"/>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A133" s="30"/>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A134" s="30"/>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A135" s="30"/>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A136" s="30"/>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A137" s="30"/>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A138" s="30"/>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A139" s="30"/>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A140" s="30"/>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A141" s="30"/>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A142" s="30"/>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A143" s="30"/>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A144" s="30"/>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A145" s="30"/>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A146" s="30"/>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A147" s="30"/>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A148" s="30"/>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A149" s="30"/>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A150" s="30"/>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A151" s="30"/>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A152" s="30"/>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A153" s="30"/>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A154" s="30"/>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A155" s="30"/>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A156" s="30"/>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A157" s="30"/>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A158" s="30"/>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A159" s="30"/>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A160" s="30"/>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A161" s="30"/>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A162" s="30"/>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A163" s="30"/>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A164" s="30"/>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A165" s="30"/>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A166" s="30"/>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A167" s="30"/>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A168" s="30"/>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A169" s="30"/>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A170" s="30"/>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A171" s="30"/>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A172" s="30"/>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A173" s="30"/>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A174" s="30"/>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A175" s="30"/>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A176" s="30"/>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A177" s="30"/>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A178" s="30"/>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A179" s="30"/>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A180" s="30"/>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A181" s="30"/>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A182" s="30"/>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A183" s="30"/>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A184" s="30"/>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A185" s="30"/>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A186" s="30"/>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A187" s="30"/>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A188" s="30"/>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A189" s="30"/>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A190" s="30"/>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A191" s="30"/>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A192" s="30"/>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A193" s="30"/>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A194" s="30"/>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A195" s="30"/>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A196" s="30"/>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A197" s="30"/>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A198" s="30"/>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A199" s="30"/>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A200" s="30"/>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A201" s="30"/>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A202" s="30"/>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A203" s="30"/>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A204" s="30"/>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A205" s="30"/>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A206" s="30"/>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A207" s="30"/>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A208" s="30"/>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A209" s="30"/>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A210" s="30"/>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A211" s="30"/>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A212" s="30"/>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A213" s="30"/>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A214" s="30"/>
+    </row>
+    <row r="215" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A215" s="30"/>
+    </row>
+    <row r="216" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A216" s="30"/>
+    </row>
+    <row r="217" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A217" s="30"/>
+    </row>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A218" s="30"/>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A219" s="30"/>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A220" s="30"/>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A221" s="30"/>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A222" s="30"/>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A223" s="30"/>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A224" s="30"/>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A225" s="30"/>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A226" s="30"/>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A227" s="30"/>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A228" s="30"/>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A229" s="30"/>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A230" s="30"/>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A231" s="30"/>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A232" s="30"/>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A233" s="30"/>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A234" s="30"/>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A235" s="30"/>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A236" s="30"/>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A237" s="30"/>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A238" s="30"/>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A239" s="30"/>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A240" s="30"/>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A241" s="30"/>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A242" s="30"/>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A243" s="30"/>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A244" s="30"/>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A245" s="30"/>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A246" s="30"/>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A247" s="30"/>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A248" s="30"/>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A249" s="30"/>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A250" s="30"/>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A251" s="30"/>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A252" s="30"/>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A253" s="30"/>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A254" s="30"/>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A255" s="30"/>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A256" s="30"/>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A257" s="30"/>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A258" s="30"/>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A259" s="30"/>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A260" s="30"/>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A261" s="30"/>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A262" s="30"/>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A263" s="30"/>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A264" s="30"/>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A265" s="30"/>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A266" s="30"/>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A267" s="30"/>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A268" s="30"/>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A269" s="30"/>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A270" s="30"/>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A271" s="30"/>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A272" s="30"/>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A273" s="30"/>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A274" s="30"/>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A275" s="30"/>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A276" s="30"/>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A277" s="30"/>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A278" s="30"/>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A279" s="30"/>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A280" s="30"/>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A281" s="30"/>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A282" s="30"/>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A283" s="30"/>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A284" s="30"/>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A285" s="30"/>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A286" s="30"/>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A287" s="30"/>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A288" s="30"/>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A289" s="30"/>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A290" s="30"/>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A291" s="30"/>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A292" s="30"/>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A293" s="30"/>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A294" s="30"/>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A295" s="30"/>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A296" s="30"/>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A297" s="30"/>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A298" s="30"/>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A299" s="30"/>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A300" s="30"/>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A301" s="30"/>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A302" s="30"/>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A303" s="30"/>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A304" s="30"/>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A305" s="30"/>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A306" s="30"/>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A307" s="30"/>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A308" s="30"/>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A309" s="30"/>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A310" s="30"/>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A311" s="30"/>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A312" s="30"/>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A313" s="30"/>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A314" s="30"/>
+    </row>
+    <row r="315" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A315" s="30"/>
+    </row>
+    <row r="316" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A316" s="30"/>
+    </row>
+    <row r="317" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A317" s="30"/>
+    </row>
+    <row r="318" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A318" s="30"/>
+    </row>
+    <row r="319" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A319" s="30"/>
+    </row>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A320" s="30"/>
+    </row>
+    <row r="321" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A321" s="30"/>
+    </row>
+    <row r="322" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A322" s="30"/>
+    </row>
+    <row r="323" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A323" s="30"/>
+    </row>
+    <row r="324" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A324" s="30"/>
+    </row>
+    <row r="325" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A325" s="30"/>
+    </row>
+    <row r="326" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A326" s="30"/>
+    </row>
+    <row r="327" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A327" s="30"/>
+    </row>
+    <row r="328" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A328" s="30"/>
+    </row>
+    <row r="329" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A329" s="30"/>
+    </row>
+    <row r="330" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A330" s="30"/>
+    </row>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A331" s="30"/>
+    </row>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A332" s="30"/>
+    </row>
+    <row r="333" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A333" s="30"/>
+    </row>
+    <row r="334" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A334" s="30"/>
+    </row>
+    <row r="335" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A335" s="30"/>
+    </row>
+    <row r="336" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A336" s="30"/>
+    </row>
+    <row r="337" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A337" s="30"/>
+    </row>
+    <row r="338" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A338" s="30"/>
+    </row>
+    <row r="339" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A339" s="30"/>
+    </row>
+    <row r="340" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A340" s="30"/>
+    </row>
+    <row r="341" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A341" s="30"/>
+    </row>
+    <row r="342" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A342" s="30"/>
+    </row>
+    <row r="343" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A343" s="30"/>
+    </row>
+    <row r="344" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A344" s="30"/>
+    </row>
+    <row r="345" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A345" s="30"/>
+    </row>
+    <row r="346" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A346" s="30"/>
+    </row>
+    <row r="347" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A347" s="30"/>
+    </row>
+    <row r="348" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A348" s="30"/>
+    </row>
+    <row r="349" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A349" s="30"/>
+    </row>
+    <row r="350" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A350" s="30"/>
+    </row>
+    <row r="351" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A351" s="30"/>
+    </row>
+    <row r="352" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A352" s="30"/>
+    </row>
+    <row r="353" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A353" s="30"/>
+    </row>
+    <row r="354" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A354" s="30"/>
+    </row>
+    <row r="355" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A355" s="30"/>
+    </row>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A356" s="30"/>
+    </row>
+    <row r="357" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A357" s="30"/>
+    </row>
+    <row r="358" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A358" s="30"/>
+    </row>
+    <row r="359" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A359" s="30"/>
+    </row>
+    <row r="360" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A360" s="30"/>
+    </row>
+    <row r="361" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A361" s="30"/>
+    </row>
+    <row r="362" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A362" s="30"/>
+    </row>
+    <row r="363" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A363" s="30"/>
+    </row>
+    <row r="364" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A364" s="30"/>
+    </row>
+    <row r="365" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A365" s="30"/>
+    </row>
+    <row r="366" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A366" s="30"/>
+    </row>
+    <row r="367" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A367" s="30"/>
+    </row>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A368" s="30"/>
+    </row>
+    <row r="369" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A369" s="30"/>
+    </row>
+    <row r="370" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A370" s="30"/>
+    </row>
+    <row r="371" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A371" s="30"/>
+    </row>
+    <row r="372" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A372" s="30"/>
+    </row>
+    <row r="373" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A373" s="30"/>
+    </row>
+    <row r="374" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A374" s="30"/>
+    </row>
+    <row r="375" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A375" s="30"/>
+    </row>
+    <row r="376" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A376" s="30"/>
+    </row>
+    <row r="377" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A377" s="30"/>
+    </row>
+    <row r="378" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A378" s="30"/>
+    </row>
+    <row r="379" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A379" s="30"/>
+    </row>
+    <row r="380" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A380" s="30"/>
+    </row>
+    <row r="381" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A381" s="30"/>
+    </row>
+    <row r="382" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A382" s="30"/>
+    </row>
+    <row r="383" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A383" s="30"/>
+    </row>
+    <row r="384" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A384" s="30"/>
+    </row>
+    <row r="385" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A385" s="30"/>
+    </row>
+    <row r="386" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A386" s="30"/>
+    </row>
+    <row r="387" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A387" s="30"/>
+    </row>
+    <row r="388" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A388" s="30"/>
+    </row>
+    <row r="389" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A389" s="30"/>
+    </row>
+    <row r="390" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A390" s="30"/>
+    </row>
+    <row r="391" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A391" s="30"/>
+    </row>
+    <row r="392" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A392" s="30"/>
+    </row>
+    <row r="393" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A393" s="30"/>
+    </row>
+    <row r="394" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A394" s="30"/>
+    </row>
+    <row r="395" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A395" s="30"/>
+    </row>
+    <row r="396" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A396" s="30"/>
+    </row>
+    <row r="397" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A397" s="30"/>
+    </row>
+    <row r="398" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A398" s="30"/>
+    </row>
+    <row r="399" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A399" s="30"/>
+    </row>
+    <row r="400" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A400" s="30"/>
+    </row>
+    <row r="401" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A401" s="30"/>
+    </row>
+    <row r="402" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A402" s="30"/>
+    </row>
+    <row r="403" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A403" s="30"/>
+    </row>
+    <row r="404" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A404" s="30"/>
+    </row>
+    <row r="405" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A405" s="30"/>
+    </row>
+    <row r="406" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A406" s="30"/>
+    </row>
+    <row r="407" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A407" s="30"/>
+    </row>
+    <row r="408" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A408" s="30"/>
+    </row>
+    <row r="409" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A409" s="30"/>
+    </row>
+    <row r="410" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A410" s="30"/>
+    </row>
+    <row r="411" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A411" s="30"/>
+    </row>
+    <row r="412" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A412" s="30"/>
+    </row>
+    <row r="413" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A413" s="30"/>
+    </row>
+    <row r="414" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A414" s="30"/>
+    </row>
+    <row r="415" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A415" s="30"/>
+    </row>
+    <row r="416" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A416" s="30"/>
+    </row>
+    <row r="417" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A417" s="30"/>
+    </row>
+    <row r="418" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A418" s="30"/>
+    </row>
+    <row r="419" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A419" s="30"/>
+    </row>
+    <row r="420" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A420" s="30"/>
+    </row>
+    <row r="421" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A421" s="30"/>
+    </row>
+    <row r="422" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A422" s="30"/>
+    </row>
+    <row r="423" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A423" s="30"/>
+    </row>
+    <row r="424" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A424" s="30"/>
+    </row>
+    <row r="425" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A425" s="30"/>
+    </row>
+    <row r="426" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A426" s="30"/>
+    </row>
+    <row r="427" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A427" s="30"/>
+    </row>
+    <row r="428" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A428" s="30"/>
+    </row>
+    <row r="429" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A429" s="30"/>
+    </row>
+    <row r="430" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A430" s="30"/>
+    </row>
+    <row r="431" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A431" s="30"/>
+    </row>
+    <row r="432" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A432" s="30"/>
+    </row>
+    <row r="433" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A433" s="30"/>
+    </row>
+    <row r="434" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A434" s="30"/>
+    </row>
+    <row r="435" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A435" s="30"/>
+    </row>
+    <row r="436" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A436" s="30"/>
+    </row>
+    <row r="437" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A437" s="30"/>
+    </row>
+    <row r="438" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A438" s="30"/>
+    </row>
+    <row r="439" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A439" s="30"/>
+    </row>
+    <row r="440" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A440" s="30"/>
+    </row>
+    <row r="441" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A441" s="30"/>
+    </row>
+    <row r="442" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A442" s="30"/>
+    </row>
+    <row r="443" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A443" s="30"/>
+    </row>
+    <row r="444" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A444" s="30"/>
+    </row>
+    <row r="445" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A445" s="30"/>
+    </row>
+    <row r="446" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A446" s="30"/>
+    </row>
+    <row r="447" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A447" s="30"/>
+    </row>
+    <row r="448" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A448" s="30"/>
+    </row>
+    <row r="449" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A449" s="30"/>
+    </row>
+    <row r="450" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A450" s="30"/>
+    </row>
+    <row r="451" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A451" s="30"/>
+    </row>
+    <row r="452" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A452" s="30"/>
+    </row>
+    <row r="453" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A453" s="30"/>
+    </row>
+    <row r="454" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A454" s="30"/>
+    </row>
+    <row r="455" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A455" s="30"/>
+    </row>
+    <row r="456" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A456" s="30"/>
+    </row>
+    <row r="457" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A457" s="30"/>
+    </row>
+    <row r="458" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A458" s="30"/>
+    </row>
+    <row r="459" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A459" s="30"/>
+    </row>
+    <row r="460" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A460" s="30"/>
+    </row>
+    <row r="461" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A461" s="30"/>
+    </row>
+    <row r="462" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A462" s="30"/>
+    </row>
+    <row r="463" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A463" s="30"/>
+    </row>
+    <row r="464" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A464" s="30"/>
+    </row>
+    <row r="465" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A465" s="30"/>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A466" s="30"/>
+    </row>
+    <row r="467" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A467" s="30"/>
+    </row>
+    <row r="468" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A468" s="30"/>
+    </row>
+    <row r="469" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A469" s="30"/>
+    </row>
+    <row r="470" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A470" s="30"/>
+    </row>
+    <row r="471" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A471" s="30"/>
+    </row>
+    <row r="472" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A472" s="30"/>
+    </row>
+    <row r="473" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A473" s="30"/>
+    </row>
+    <row r="474" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A474" s="30"/>
+    </row>
+    <row r="475" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A475" s="30"/>
+    </row>
+    <row r="476" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A476" s="30"/>
+    </row>
+    <row r="477" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A477" s="30"/>
+    </row>
+    <row r="478" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A478" s="30"/>
+    </row>
+    <row r="479" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A479" s="30"/>
+    </row>
+    <row r="480" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A480" s="30"/>
+    </row>
+    <row r="481" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A481" s="30"/>
+    </row>
+    <row r="482" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A482" s="30"/>
+    </row>
+    <row r="483" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A483" s="30"/>
+    </row>
+    <row r="484" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A484" s="30"/>
+    </row>
+    <row r="485" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A485" s="30"/>
+    </row>
+    <row r="486" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A486" s="30"/>
+    </row>
+    <row r="487" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A487" s="30"/>
+    </row>
+    <row r="488" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A488" s="30"/>
+    </row>
+    <row r="489" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A489" s="30"/>
+    </row>
+    <row r="490" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A490" s="30"/>
+    </row>
+    <row r="491" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A491" s="30"/>
+    </row>
+    <row r="492" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A492" s="30"/>
+    </row>
+    <row r="493" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A493" s="30"/>
+    </row>
+    <row r="494" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A494" s="30"/>
+    </row>
+    <row r="495" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A495" s="30"/>
+    </row>
+    <row r="496" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A496" s="30"/>
+    </row>
+    <row r="497" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A497" s="30"/>
+    </row>
+    <row r="498" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A498" s="30"/>
+    </row>
+    <row r="499" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A499" s="30"/>
+    </row>
+    <row r="500" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A500" s="30"/>
+    </row>
+    <row r="501" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A501" s="30"/>
+    </row>
+    <row r="502" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A502" s="30"/>
+    </row>
+    <row r="503" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A503" s="30"/>
+    </row>
+    <row r="504" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A504" s="30"/>
+    </row>
+    <row r="505" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A505" s="30"/>
+    </row>
+    <row r="506" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A506" s="30"/>
+    </row>
+    <row r="507" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A507" s="30"/>
+    </row>
+    <row r="508" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A508" s="30"/>
+    </row>
+    <row r="509" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A509" s="30"/>
+    </row>
+    <row r="510" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A510" s="30"/>
+    </row>
+    <row r="511" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A511" s="30"/>
+    </row>
+    <row r="512" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A512" s="30"/>
+    </row>
+    <row r="513" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A513" s="30"/>
+    </row>
+    <row r="514" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A514" s="30"/>
+    </row>
+    <row r="515" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A515" s="30"/>
+    </row>
+    <row r="516" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A516" s="30"/>
+    </row>
+    <row r="517" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A517" s="30"/>
+    </row>
+    <row r="518" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A518" s="30"/>
+    </row>
+    <row r="519" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A519" s="30"/>
+    </row>
+    <row r="520" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A520" s="30"/>
+    </row>
+    <row r="521" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A521" s="30"/>
+    </row>
+    <row r="522" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A522" s="30"/>
+    </row>
+    <row r="523" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A523" s="30"/>
+    </row>
+    <row r="524" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A524" s="30"/>
+    </row>
+    <row r="525" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A525" s="30"/>
+    </row>
+    <row r="526" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A526" s="30"/>
+    </row>
+    <row r="527" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A527" s="30"/>
+    </row>
+    <row r="528" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A528" s="30"/>
+    </row>
+    <row r="529" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A529" s="30"/>
+    </row>
+    <row r="530" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A530" s="30"/>
+    </row>
+    <row r="531" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A531" s="30"/>
+    </row>
+    <row r="532" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A532" s="30"/>
+    </row>
+    <row r="533" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A533" s="30"/>
+    </row>
+    <row r="534" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A534" s="30"/>
+    </row>
+    <row r="535" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A535" s="30"/>
+    </row>
+    <row r="536" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A536" s="30"/>
+    </row>
+    <row r="537" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A537" s="30"/>
+    </row>
+    <row r="538" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A538" s="30"/>
+    </row>
+    <row r="539" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A539" s="30"/>
+    </row>
+    <row r="540" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A540" s="30"/>
+    </row>
+    <row r="541" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A541" s="30"/>
+    </row>
+    <row r="542" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A542" s="30"/>
+    </row>
+    <row r="543" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A543" s="30"/>
+    </row>
+    <row r="544" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A544" s="30"/>
+    </row>
+    <row r="545" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A545" s="30"/>
+    </row>
+    <row r="546" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A546" s="30"/>
+    </row>
+    <row r="547" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A547" s="30"/>
+    </row>
+    <row r="548" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A548" s="30"/>
+    </row>
+    <row r="549" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A549" s="30"/>
+    </row>
+    <row r="550" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A550" s="30"/>
+    </row>
+    <row r="551" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A551" s="30"/>
+    </row>
+    <row r="552" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A552" s="30"/>
+    </row>
+    <row r="553" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A553" s="30"/>
+    </row>
+    <row r="554" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A554" s="30"/>
+    </row>
+    <row r="555" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A555" s="30"/>
+    </row>
+    <row r="556" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A556" s="30"/>
+    </row>
+    <row r="557" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A557" s="30"/>
+    </row>
+    <row r="558" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A558" s="30"/>
+    </row>
+    <row r="559" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A559" s="30"/>
+    </row>
+    <row r="560" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A560" s="30"/>
+    </row>
+    <row r="561" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A561" s="30"/>
+    </row>
+    <row r="562" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A562" s="30"/>
+    </row>
+    <row r="563" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A563" s="30"/>
+    </row>
+    <row r="564" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A564" s="30"/>
+    </row>
+    <row r="565" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A565" s="30"/>
+    </row>
+    <row r="566" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A566" s="30"/>
+    </row>
+    <row r="567" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A567" s="30"/>
+    </row>
+    <row r="568" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A568" s="30"/>
+    </row>
+    <row r="569" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A569" s="30"/>
+    </row>
+    <row r="570" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A570" s="30"/>
+    </row>
+    <row r="571" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A571" s="30"/>
+    </row>
+    <row r="572" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A572" s="30"/>
+    </row>
+    <row r="573" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A573" s="30"/>
+    </row>
+    <row r="574" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A574" s="30"/>
+    </row>
+    <row r="575" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A575" s="30"/>
+    </row>
+    <row r="576" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A576" s="30"/>
+    </row>
+    <row r="577" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A577" s="30"/>
+    </row>
+    <row r="578" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A578" s="30"/>
+    </row>
+    <row r="579" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A579" s="30"/>
+    </row>
+    <row r="580" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A580" s="30"/>
+    </row>
+    <row r="581" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A581" s="30"/>
+    </row>
+    <row r="582" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A582" s="30"/>
+    </row>
+    <row r="583" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A583" s="30"/>
+    </row>
+    <row r="584" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A584" s="30"/>
+    </row>
+    <row r="585" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A585" s="30"/>
+    </row>
+    <row r="586" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A586" s="30"/>
+    </row>
+    <row r="587" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A587" s="30"/>
+    </row>
+    <row r="588" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A588" s="30"/>
+    </row>
+    <row r="589" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A589" s="30"/>
+    </row>
+    <row r="590" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A590" s="30"/>
+    </row>
+    <row r="591" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A591" s="30"/>
+    </row>
+    <row r="592" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A592" s="30"/>
+    </row>
+    <row r="593" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A593" s="30"/>
+    </row>
+    <row r="594" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A594" s="30"/>
+    </row>
+    <row r="595" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A595" s="30"/>
+    </row>
+    <row r="596" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A596" s="30"/>
+    </row>
+    <row r="597" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A597" s="30"/>
+    </row>
+    <row r="598" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A598" s="30"/>
+    </row>
+    <row r="599" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A599" s="30"/>
+    </row>
+    <row r="600" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A600" s="30"/>
+    </row>
+    <row r="601" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A601" s="30"/>
+    </row>
+    <row r="602" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A602" s="30"/>
+    </row>
+    <row r="603" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A603" s="30"/>
+    </row>
+    <row r="604" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A604" s="30"/>
+    </row>
+    <row r="605" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A605" s="30"/>
+    </row>
+    <row r="606" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A606" s="30"/>
+    </row>
+    <row r="607" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A607" s="30"/>
+    </row>
+    <row r="608" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A608" s="30"/>
+    </row>
+    <row r="609" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A609" s="30"/>
+    </row>
+    <row r="610" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A610" s="30"/>
+    </row>
+    <row r="611" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A611" s="30"/>
+    </row>
+    <row r="612" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A612" s="30"/>
+    </row>
+    <row r="613" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A613" s="30"/>
+    </row>
+    <row r="614" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A614" s="30"/>
+    </row>
+    <row r="615" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A615" s="30"/>
+    </row>
+    <row r="616" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A616" s="30"/>
+    </row>
+    <row r="617" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A617" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates for HST data to use common plotting tools
</commit_message>
<xml_diff>
--- a/Catalog/Catalog-static.xlsx
+++ b/Catalog/Catalog-static.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Astronomy\Projects\SAS 2021 Ammonia\Jupiter_NH3_Analysis_P3\Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E58B082-47C5-4462-AB28-2DEDC0A213F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25446C97-6415-4CBB-BD6C-0028DA54D7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5887" uniqueCount="2457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5903" uniqueCount="2467">
   <si>
     <t>ObsID</t>
   </si>
@@ -7474,9 +7474,6 @@
     <t>Some clouds, appears to be clearing (some clouds throughout the night?). Seeing  was very good to excellent. Last sequence may be contaminated by twilight. Moons?</t>
   </si>
   <si>
-    <t>Very clear, fair seeing</t>
-  </si>
-  <si>
     <t>Very clear. Good seeing once Jupiter was high enough above the horizon</t>
   </si>
   <si>
@@ -7515,9 +7512,6 @@
       </rPr>
       <t xml:space="preserve"> possibly the best seeing this apparition</t>
     </r>
-  </si>
-  <si>
-    <t>Very clear and pretty good (maybe fair to poor) seeing</t>
   </si>
   <si>
     <r>
@@ -7549,7 +7543,212 @@
     <t>Good seeing. Clear, then clouds came in</t>
   </si>
   <si>
-    <t>Very good seeing. Very transparent. Extraordinary seeing in the middle of the night. Maybe 24 of 27 are very good quality.</t>
+    <r>
+      <t xml:space="preserve">Very good seeing. Very transparent. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Extraordinary seeing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>in the middle of the night. Maybe 24 of 27 are very good quality.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Extraordinary seeing, maybe best of season. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Very clear</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Extraordinary seeing, one of the best of season. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Very clear</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Very clear, fair seeing; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>HST</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> imaging on 12/21</t>
+    </r>
+  </si>
+  <si>
+    <t>Very good seeing. Good transparency, then clouded out</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SEB outbreak! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Very good seeing, Fair to poor transparency 2/5 high haze</t>
+    </r>
+  </si>
+  <si>
+    <t>Very good seeing. Transparency fair with high, thin cirrus</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Excellent seeing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, very good transparency. Lost about 40 mins at ~9:10 due to some anomalous pointing error, need to check logs</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Excellent seeing.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Transparency good until clouded out</t>
+    </r>
+  </si>
+  <si>
+    <t>Very good seeing. Excellent transparency. Should have good coverage of SEB outbreak. Got a bit of a late start - had to wait for havdallah</t>
+  </si>
+  <si>
+    <r>
+      <t>Very clear and pretty good (maybe fair to poor) seeing -</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>May have processed only 26 files due to limit of alphabet</t>
+    </r>
+  </si>
+  <si>
+    <t>Processed V1</t>
+  </si>
+  <si>
+    <t>Processed V2</t>
   </si>
 </sst>
 </file>
@@ -8170,7 +8369,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -8270,8 +8469,9 @@
     </xf>
     <xf numFmtId="165" fontId="16" fillId="46" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="46" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="47" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="47" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -40383,7 +40583,7 @@
       </c>
       <c r="B1" s="18">
         <f>SUM(B2:B151)</f>
-        <v>1135</v>
+        <v>1303</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>696</v>
@@ -40402,10 +40602,10 @@
       <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40416,10 +40616,10 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40430,10 +40630,10 @@
       <c r="B4">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40444,10 +40644,10 @@
       <c r="B5">
         <v>2</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40458,10 +40658,10 @@
       <c r="B6">
         <v>2</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40472,10 +40672,10 @@
       <c r="B7">
         <v>2</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40486,10 +40686,10 @@
       <c r="B8">
         <v>2</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40500,10 +40700,10 @@
       <c r="B9">
         <v>3</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40514,10 +40714,10 @@
       <c r="B10">
         <v>2</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40528,10 +40728,10 @@
       <c r="B11">
         <v>2</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40542,10 +40742,10 @@
       <c r="B12">
         <v>2</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40556,10 +40756,10 @@
       <c r="B13">
         <v>2</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40570,10 +40770,10 @@
       <c r="B14">
         <v>2</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40584,10 +40784,10 @@
       <c r="B15">
         <v>1</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -40598,10 +40798,10 @@
       <c r="B16">
         <v>10</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E16" t="s">
@@ -40615,10 +40815,10 @@
       <c r="B17">
         <v>10</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E17" t="s">
@@ -40632,7 +40832,7 @@
       <c r="B18">
         <v>11</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="57" t="s">
         <v>687</v>
       </c>
       <c r="D18" s="33" t="s">
@@ -40649,10 +40849,10 @@
       <c r="B19">
         <v>9</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E19" t="s">
@@ -40666,10 +40866,10 @@
       <c r="B20">
         <v>16</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E20" t="s">
@@ -40683,7 +40883,7 @@
       <c r="B21">
         <v>15</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="57" t="s">
         <v>687</v>
       </c>
       <c r="D21" s="33" t="s">
@@ -40700,7 +40900,7 @@
       <c r="B22">
         <v>11</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="57" t="s">
         <v>687</v>
       </c>
       <c r="D22" s="33" t="s">
@@ -40717,10 +40917,10 @@
       <c r="B23">
         <v>14</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E23" t="s">
@@ -40734,10 +40934,10 @@
       <c r="B24">
         <v>14</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E24" t="s">
@@ -40751,10 +40951,10 @@
       <c r="B25">
         <v>8</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E25" t="s">
@@ -40768,10 +40968,10 @@
       <c r="B26">
         <v>16</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E26" t="s">
@@ -40785,10 +40985,10 @@
       <c r="B27">
         <v>17</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E27" t="s">
@@ -40802,10 +41002,10 @@
       <c r="B28">
         <v>4</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E28" t="s">
@@ -40819,10 +41019,10 @@
       <c r="B29">
         <v>20</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E29" t="s">
@@ -40839,7 +41039,7 @@
       <c r="C30" s="9" t="s">
         <v>687</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E30" t="s">
@@ -40867,10 +41067,10 @@
       <c r="B32">
         <v>21</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E32" t="s">
@@ -40884,10 +41084,10 @@
       <c r="B33">
         <v>20</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E33" t="s">
@@ -40901,10 +41101,10 @@
       <c r="B34">
         <v>16</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E34" t="s">
@@ -40918,10 +41118,10 @@
       <c r="B35">
         <v>19</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E35" t="s">
@@ -40935,10 +41135,10 @@
       <c r="B36">
         <v>19</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="57" t="s">
         <v>695</v>
       </c>
       <c r="E36" t="s">
@@ -40977,7 +41177,7 @@
       <c r="B39">
         <v>6</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="57" t="s">
         <v>687</v>
       </c>
       <c r="D39" s="9" t="s">
@@ -40994,7 +41194,7 @@
       <c r="B40">
         <v>9</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="57" t="s">
         <v>687</v>
       </c>
       <c r="D40" s="9" t="s">
@@ -41008,10 +41208,10 @@
       <c r="B41">
         <v>9</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="57" t="s">
         <v>695</v>
       </c>
     </row>
@@ -41022,7 +41222,7 @@
       <c r="B42">
         <v>7</v>
       </c>
-      <c r="D42" s="57" t="s">
+      <c r="D42" s="59" t="s">
         <v>695</v>
       </c>
     </row>
@@ -41033,7 +41233,7 @@
       <c r="B43">
         <v>6</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="57" t="s">
         <v>687</v>
       </c>
       <c r="D43" s="33" t="s">
@@ -41050,11 +41250,11 @@
       <c r="B44">
         <v>6</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D44" t="s">
-        <v>695</v>
+      <c r="D44" s="57" t="s">
+        <v>2465</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
@@ -41064,11 +41264,11 @@
       <c r="B45">
         <v>7</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D45" t="s">
-        <v>695</v>
+      <c r="D45" s="57" t="s">
+        <v>2465</v>
       </c>
       <c r="E45" t="s">
         <v>1832</v>
@@ -41081,11 +41281,11 @@
       <c r="B46">
         <v>7</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D46" t="s">
-        <v>695</v>
+      <c r="D46" s="57" t="s">
+        <v>2465</v>
       </c>
       <c r="E46" t="s">
         <v>1832</v>
@@ -41098,11 +41298,11 @@
       <c r="B47">
         <v>9</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D47" t="s">
-        <v>695</v>
+      <c r="D47" s="57" t="s">
+        <v>2465</v>
       </c>
       <c r="E47" t="s">
         <v>1831</v>
@@ -41115,11 +41315,11 @@
       <c r="B48">
         <v>9</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D48" t="s">
-        <v>695</v>
+      <c r="D48" s="57" t="s">
+        <v>2465</v>
       </c>
       <c r="E48" t="s">
         <v>1831</v>
@@ -41132,8 +41332,11 @@
       <c r="B49">
         <v>11</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="57" t="s">
         <v>687</v>
+      </c>
+      <c r="D49" s="51" t="s">
+        <v>2450</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
@@ -41151,11 +41354,11 @@
       <c r="B51">
         <v>14</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D51" s="51" t="s">
-        <v>695</v>
+      <c r="D51" s="57" t="s">
+        <v>2465</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
@@ -41165,11 +41368,11 @@
       <c r="B52">
         <v>12</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C52" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D52" s="51" t="s">
-        <v>695</v>
+      <c r="D52" s="57" t="s">
+        <v>2465</v>
       </c>
       <c r="E52" t="s">
         <v>2045</v>
@@ -41182,11 +41385,11 @@
       <c r="B53">
         <v>15</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C53" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D53" s="51" t="s">
-        <v>695</v>
+      <c r="D53" s="57" t="s">
+        <v>2465</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
@@ -41196,8 +41399,11 @@
       <c r="B54">
         <v>16</v>
       </c>
-      <c r="D54" s="51" t="s">
-        <v>695</v>
+      <c r="C54" s="57" t="s">
+        <v>687</v>
+      </c>
+      <c r="D54" s="57" t="s">
+        <v>2466</v>
       </c>
       <c r="E54" t="s">
         <v>2048</v>
@@ -41309,8 +41515,11 @@
       <c r="B64">
         <v>21</v>
       </c>
-      <c r="D64" s="51" t="s">
-        <v>695</v>
+      <c r="C64" s="57" t="s">
+        <v>687</v>
+      </c>
+      <c r="D64" s="57" t="s">
+        <v>2466</v>
       </c>
       <c r="E64" s="18" t="s">
         <v>2441</v>
@@ -41323,8 +41532,11 @@
       <c r="B65">
         <v>20</v>
       </c>
-      <c r="D65" s="51" t="s">
-        <v>695</v>
+      <c r="C65" s="57" t="s">
+        <v>687</v>
+      </c>
+      <c r="D65" s="57" t="s">
+        <v>2465</v>
       </c>
       <c r="E65" t="s">
         <v>2442</v>
@@ -41426,11 +41638,14 @@
         <f>198/22</f>
         <v>9</v>
       </c>
-      <c r="D74" s="58" t="s">
+      <c r="C74" s="57" t="s">
+        <v>687</v>
+      </c>
+      <c r="D74" s="57" t="s">
+        <v>2466</v>
+      </c>
+      <c r="E74" s="18" t="s">
         <v>2451</v>
-      </c>
-      <c r="E74" s="18" t="s">
-        <v>2452</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
@@ -41440,11 +41655,14 @@
       <c r="B75">
         <v>27</v>
       </c>
-      <c r="D75" s="58" t="s">
-        <v>2451</v>
+      <c r="C75" s="57" t="s">
+        <v>687</v>
+      </c>
+      <c r="D75" s="57" t="s">
+        <v>2466</v>
       </c>
       <c r="E75" t="s">
-        <v>2453</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
@@ -41454,11 +41672,11 @@
       <c r="B76">
         <v>19</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C76" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D76" s="58" t="s">
-        <v>2451</v>
+      <c r="D76" s="57" t="s">
+        <v>2466</v>
       </c>
       <c r="E76" t="s">
         <v>2438</v>
@@ -41471,14 +41689,14 @@
       <c r="B77">
         <v>28</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C77" s="57" t="s">
         <v>687</v>
       </c>
-      <c r="D77" s="58" t="s">
-        <v>2451</v>
+      <c r="D77" s="57" t="s">
+        <v>2466</v>
       </c>
       <c r="E77" t="s">
-        <v>2443</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
@@ -41488,9 +41706,14 @@
       <c r="B78">
         <v>26</v>
       </c>
-      <c r="D78" s="58"/>
+      <c r="C78" s="57" t="s">
+        <v>687</v>
+      </c>
+      <c r="D78" s="51" t="s">
+        <v>2450</v>
+      </c>
       <c r="E78" t="s">
-        <v>2444</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
@@ -41500,11 +41723,11 @@
       <c r="B79">
         <v>27</v>
       </c>
-      <c r="D79" s="58" t="s">
-        <v>2451</v>
+      <c r="D79" s="51" t="s">
+        <v>2450</v>
       </c>
       <c r="E79" t="s">
-        <v>2454</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
@@ -41514,9 +41737,9 @@
       <c r="B80">
         <v>28</v>
       </c>
-      <c r="D80" s="51"/>
+      <c r="D80" s="58"/>
       <c r="E80" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
@@ -41527,7 +41750,7 @@
         <v>26</v>
       </c>
       <c r="E81" t="s">
-        <v>2446</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
@@ -41538,7 +41761,7 @@
         <v>26</v>
       </c>
       <c r="E82" t="s">
-        <v>2447</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
@@ -41549,7 +41772,7 @@
         <v>27</v>
       </c>
       <c r="E83" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
@@ -41560,7 +41783,7 @@
         <v>23</v>
       </c>
       <c r="E84" t="s">
-        <v>2448</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
@@ -41571,7 +41794,7 @@
         <v>28</v>
       </c>
       <c r="E85" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
@@ -41582,7 +41805,7 @@
         <v>26</v>
       </c>
       <c r="E86" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
@@ -41593,7 +41816,7 @@
         <v>18</v>
       </c>
       <c r="E87" t="s">
-        <v>2455</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
@@ -41604,32 +41827,96 @@
         <v>27</v>
       </c>
       <c r="E88" t="s">
+        <v>2454</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A89" s="30">
+        <v>46052</v>
+      </c>
+      <c r="B89">
+        <v>27</v>
+      </c>
+      <c r="E89" t="s">
+        <v>2455</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A90" s="30">
+        <v>46054</v>
+      </c>
+      <c r="B90">
+        <v>24</v>
+      </c>
+      <c r="E90" t="s">
         <v>2456</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A89" s="30"/>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90" s="30"/>
-    </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A91" s="30"/>
+      <c r="A91" s="30">
+        <v>46056</v>
+      </c>
+      <c r="B91">
+        <v>18</v>
+      </c>
+      <c r="E91" t="s">
+        <v>2458</v>
+      </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A92" s="30"/>
+      <c r="A92" s="30">
+        <v>46058</v>
+      </c>
+      <c r="B92">
+        <v>26</v>
+      </c>
+      <c r="E92" t="s">
+        <v>2459</v>
+      </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A93" s="30"/>
+      <c r="A93" s="30">
+        <v>46059</v>
+      </c>
+      <c r="B93">
+        <v>25</v>
+      </c>
+      <c r="E93" t="s">
+        <v>2460</v>
+      </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A94" s="30"/>
+      <c r="A94" s="30">
+        <v>46061</v>
+      </c>
+      <c r="B94">
+        <v>20</v>
+      </c>
+      <c r="E94" t="s">
+        <v>2461</v>
+      </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="30"/>
+      <c r="A95" s="30">
+        <v>46062</v>
+      </c>
+      <c r="B95">
+        <v>9</v>
+      </c>
+      <c r="E95" t="s">
+        <v>2462</v>
+      </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A96" s="30"/>
+      <c r="A96" s="30">
+        <v>46068</v>
+      </c>
+      <c r="B96">
+        <v>19</v>
+      </c>
+      <c r="E96" t="s">
+        <v>2463</v>
+      </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" s="30"/>

</xml_diff>

<commit_message>
Interim Commit - next should be a branch!
Partial integration of L3 and L4 plotting routines, along with HST data, complete. However, Rossby wave longitudinal profile plots are currently broken
</commit_message>
<xml_diff>
--- a/Catalog/Catalog-static.xlsx
+++ b/Catalog/Catalog-static.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Astronomy\Projects\SAS 2021 Ammonia\Jupiter_NH3_Analysis_P3\Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CBF7533-38BC-466C-B311-CC5DB8014B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE030F45-5AB2-41CE-B6B5-ACD91A0A75DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5924" uniqueCount="2471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5953" uniqueCount="2481">
   <si>
     <t>ObsID</t>
   </si>
@@ -7765,9 +7765,6 @@
     <t>Very good seeing. Very clear, maybe high clouds later. Sequence stopped on NIR on the 15th sequence (incomplete) for unknown reasons. Should have gone to 17</t>
   </si>
   <si>
-    <t>Excellent seeing. Very clear.</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Very good seeing. Very transparent. </t>
     </r>
@@ -7823,6 +7820,52 @@
   </si>
   <si>
     <t>Good seeing, very good transparency. Took three observations while still twilight, can see how they turned out</t>
+  </si>
+  <si>
+    <t>DeTeCt Run?</t>
+  </si>
+  <si>
+    <t>Fair seeing, excellent transparency (missing one settings file, 351 total)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Fair seeing, excellent transparency, missed about 25 minutes due to a late flip (time change messed me up?), MOON &amp; SHADOW</t>
+  </si>
+  <si>
+    <t>Fair seeing, fair transparency (some high, thin clouds at dusk)</t>
+  </si>
+  <si>
+    <t>1 Low</t>
+  </si>
+  <si>
+    <t>2 Low</t>
+  </si>
+  <si>
+    <t>Fair to poor seeing, good transparency</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Excellent seeing. Very clear. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Some of the last images are dim and have problems stacking. Need to fix this. Did manual registax 5 for IGB</t>
+    </r>
+  </si>
+  <si>
+    <t>I THINK I HAVE ALL THE DeTeCt ZIP FILES, BUT I NEED TO REVIEW THEM INDIVIDUALLY BEFORE UPLOADING</t>
+  </si>
+  <si>
+    <t>I ALSO NEED TO RECOMBINE THE 3/8/2026 FILES ON THE ARCHIVE DRIVE - I ACCIDENTALLY MOVED A BUNCH OFF INSTEAD OF COPYING THEM</t>
   </si>
 </sst>
 </file>
@@ -8005,7 +8048,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="50">
+  <fills count="51">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8287,8 +8330,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF48484"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -8403,6 +8452,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -8448,7 +8534,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -8551,6 +8637,12 @@
     <xf numFmtId="0" fontId="0" fillId="46" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="48" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="49" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="41" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="41" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="41" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -8598,6 +8690,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF48484"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -40646,23 +40743,24 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FB822E-4FB0-4362-8846-871BD8F7A1EF}">
-  <dimension ref="A1:I617"/>
+  <dimension ref="A1:J617"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
     <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.81640625" customWidth="1"/>
     <col min="4" max="4" width="12.7265625" customWidth="1"/>
-    <col min="5" max="5" width="47.54296875" customWidth="1"/>
+    <col min="5" max="5" width="10.7265625" customWidth="1"/>
+    <col min="6" max="6" width="47.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" s="18" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="31" t="s">
         <v>685</v>
       </c>
       <c r="B1" s="18">
         <f>SUM(B2:B151)</f>
-        <v>1379</v>
+        <v>1441</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>695</v>
@@ -40671,10 +40769,13 @@
         <v>686</v>
       </c>
       <c r="E1" s="18" t="s">
+        <v>2470</v>
+      </c>
+      <c r="F1" s="18" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="30">
         <v>45554</v>
       </c>
@@ -40688,7 +40789,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="30">
         <v>45558</v>
       </c>
@@ -40702,7 +40803,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="30">
         <v>45560</v>
       </c>
@@ -40716,7 +40817,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="30">
         <v>45564</v>
       </c>
@@ -40730,7 +40831,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="30">
         <v>45567</v>
       </c>
@@ -40744,7 +40845,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="30">
         <v>45571</v>
       </c>
@@ -40758,7 +40859,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="30">
         <v>45572</v>
       </c>
@@ -40772,7 +40873,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="30">
         <v>45573</v>
       </c>
@@ -40786,7 +40887,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="30">
         <v>45574</v>
       </c>
@@ -40800,7 +40901,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="30">
         <v>45575</v>
       </c>
@@ -40814,7 +40915,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="30">
         <v>45579</v>
       </c>
@@ -40828,7 +40929,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="30">
         <v>45581</v>
       </c>
@@ -40842,7 +40943,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="30">
         <v>45587</v>
       </c>
@@ -40856,7 +40957,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="30">
         <v>45588</v>
       </c>
@@ -40870,7 +40971,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="30">
         <v>45592</v>
       </c>
@@ -40883,11 +40984,11 @@
       <c r="D16" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>913</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="30">
         <v>45601</v>
       </c>
@@ -40900,11 +41001,11 @@
       <c r="D17" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>914</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="30">
         <v>45607</v>
       </c>
@@ -40917,11 +41018,11 @@
       <c r="D18" s="57" t="s">
         <v>2446</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>1825</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="30">
         <v>45611</v>
       </c>
@@ -40934,11 +41035,11 @@
       <c r="D19" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>915</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="30">
         <v>45614</v>
       </c>
@@ -40951,11 +41052,11 @@
       <c r="D20" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>909</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="30">
         <v>45617</v>
       </c>
@@ -40968,11 +41069,11 @@
       <c r="D21" s="58" t="s">
         <v>2446</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>910</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="30">
         <v>45620</v>
       </c>
@@ -40985,11 +41086,11 @@
       <c r="D22" s="58" t="s">
         <v>2446</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>910</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="30">
         <v>45624</v>
       </c>
@@ -41002,11 +41103,11 @@
       <c r="D23" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>916</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="30">
         <v>45625</v>
       </c>
@@ -41019,11 +41120,11 @@
       <c r="D24" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>907</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="30">
         <v>45628</v>
       </c>
@@ -41036,11 +41137,11 @@
       <c r="D25" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>907</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="30">
         <v>45629</v>
       </c>
@@ -41053,11 +41154,11 @@
       <c r="D26" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E26" t="s">
+      <c r="F26" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="30">
         <v>45631</v>
       </c>
@@ -41070,11 +41171,11 @@
       <c r="D27" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E27" t="s">
+      <c r="F27" t="s">
         <v>917</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="30">
         <v>45657</v>
       </c>
@@ -41087,11 +41188,11 @@
       <c r="D28" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" t="s">
         <v>1559</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="30">
         <v>45663</v>
       </c>
@@ -41104,11 +41205,11 @@
       <c r="D29" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>1558</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="30">
         <v>45671</v>
       </c>
@@ -41121,11 +41222,11 @@
       <c r="D30" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>1554</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="30">
         <v>45672</v>
       </c>
@@ -41135,11 +41236,12 @@
       <c r="D31" s="32" t="s">
         <v>1557</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="32"/>
+      <c r="F31" t="s">
         <v>1555</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="30">
         <v>45673</v>
       </c>
@@ -41152,11 +41254,11 @@
       <c r="D32" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>1556</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="30">
         <v>45674</v>
       </c>
@@ -41169,11 +41271,11 @@
       <c r="D33" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>1826</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="30">
         <v>45684</v>
       </c>
@@ -41186,11 +41288,11 @@
       <c r="D34" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>918</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="30">
         <v>45685</v>
       </c>
@@ -41203,11 +41305,11 @@
       <c r="D35" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>908</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="30">
         <v>45686</v>
       </c>
@@ -41220,11 +41322,11 @@
       <c r="D36" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>912</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="30">
         <v>45688</v>
       </c>
@@ -41234,22 +41336,22 @@
       <c r="D37" s="50" t="s">
         <v>2446</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>1553</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="30">
         <v>45695</v>
       </c>
       <c r="B38">
         <v>17</v>
       </c>
-      <c r="E38" t="s">
+      <c r="F38" t="s">
         <v>1553</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="30">
         <v>45715</v>
       </c>
@@ -41262,11 +41364,11 @@
       <c r="D39" s="59" t="s">
         <v>2446</v>
       </c>
-      <c r="E39" t="s">
-        <v>2469</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F39" t="s">
+        <v>2468</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="30">
         <v>45716</v>
       </c>
@@ -41280,7 +41382,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="30">
         <v>45718</v>
       </c>
@@ -41294,7 +41396,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="30">
         <v>45725</v>
       </c>
@@ -41302,13 +41404,13 @@
         <v>7</v>
       </c>
       <c r="C42" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
       <c r="D42" s="56" t="s">
         <v>2459</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="30">
         <v>45726</v>
       </c>
@@ -41322,7 +41424,7 @@
         <v>2460</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="30">
         <v>45919</v>
       </c>
@@ -41336,7 +41438,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="30">
         <v>45925</v>
       </c>
@@ -41349,11 +41451,11 @@
       <c r="D45" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>1828</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="30">
         <v>45926</v>
       </c>
@@ -41366,11 +41468,11 @@
       <c r="D46" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>1828</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="30">
         <v>45930</v>
       </c>
@@ -41383,11 +41485,11 @@
       <c r="D47" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>1827</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="30">
         <v>45931</v>
       </c>
@@ -41400,11 +41502,11 @@
       <c r="D48" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>1827</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="30">
         <v>45939</v>
       </c>
@@ -41418,7 +41520,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="30">
         <v>45942</v>
       </c>
@@ -41426,7 +41528,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="30">
         <v>45946</v>
       </c>
@@ -41440,7 +41542,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="30">
         <v>45947</v>
       </c>
@@ -41453,11 +41555,11 @@
       <c r="D52" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
         <v>2041</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="30">
         <v>45949</v>
       </c>
@@ -41471,7 +41573,7 @@
         <v>2459</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="30">
         <v>45950</v>
       </c>
@@ -41484,110 +41586,110 @@
       <c r="D54" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>2044</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="30">
         <v>45959</v>
       </c>
       <c r="B55">
         <v>18</v>
       </c>
-      <c r="E55" t="s">
+      <c r="F55" t="s">
         <v>2042</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="30">
         <v>45960</v>
       </c>
       <c r="B56">
         <v>10</v>
       </c>
-      <c r="E56" t="s">
+      <c r="F56" t="s">
         <v>2043</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="30">
         <v>45963</v>
       </c>
       <c r="B57">
         <v>20</v>
       </c>
-      <c r="E57" t="s">
+      <c r="F57" t="s">
         <v>2045</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="30">
         <v>45964</v>
       </c>
       <c r="B58">
         <v>20</v>
       </c>
-      <c r="E58" t="s">
+      <c r="F58" t="s">
         <v>2436</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="30">
         <v>45965</v>
       </c>
       <c r="B59">
         <v>13</v>
       </c>
-      <c r="E59" t="s">
+      <c r="F59" t="s">
         <v>2435</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="30">
         <v>45966</v>
       </c>
       <c r="B60">
         <v>4</v>
       </c>
-      <c r="E60" t="s">
+      <c r="F60" t="s">
         <v>2200</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="30">
         <v>45971</v>
       </c>
       <c r="B61">
         <v>20</v>
       </c>
-      <c r="E61" t="s">
+      <c r="F61" t="s">
         <v>2201</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="30">
         <v>45973</v>
       </c>
       <c r="B62">
         <v>11</v>
       </c>
-      <c r="E62" t="s">
+      <c r="F62" t="s">
         <v>2202</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="30">
         <v>45975</v>
       </c>
       <c r="B63">
         <v>11</v>
       </c>
-      <c r="E63" t="s">
+      <c r="F63" t="s">
         <v>2425</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="30">
         <v>45977</v>
       </c>
@@ -41600,11 +41702,11 @@
       <c r="D64" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E64" s="18" t="s">
+      <c r="F64" s="18" t="s">
         <v>2437</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="30">
         <v>45980</v>
       </c>
@@ -41617,99 +41719,99 @@
       <c r="D65" s="56" t="s">
         <v>2459</v>
       </c>
-      <c r="E65" t="s">
+      <c r="F65" t="s">
         <v>2438</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="30">
         <v>45984</v>
       </c>
       <c r="B66">
         <v>9</v>
       </c>
-      <c r="E66" t="s">
+      <c r="F66" t="s">
         <v>2427</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" s="30">
         <v>45986</v>
       </c>
       <c r="B67">
         <v>4</v>
       </c>
-      <c r="E67" t="s">
+      <c r="F67" t="s">
         <v>2428</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="30">
         <v>45987</v>
       </c>
       <c r="B68">
         <v>17</v>
       </c>
-      <c r="E68" t="s">
+      <c r="F68" t="s">
         <v>2426</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="30">
         <v>45988</v>
       </c>
       <c r="B69">
         <v>16</v>
       </c>
-      <c r="E69" t="s">
+      <c r="F69" t="s">
         <v>2429</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" s="30">
         <v>45993</v>
       </c>
       <c r="B70">
         <v>14</v>
       </c>
-      <c r="E70" t="s">
+      <c r="F70" t="s">
         <v>2431</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" s="30">
         <v>45998</v>
       </c>
       <c r="B71">
         <v>23</v>
       </c>
-      <c r="E71" t="s">
+      <c r="F71" t="s">
         <v>2430</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="30">
         <v>46000</v>
       </c>
       <c r="B72">
         <v>4</v>
       </c>
-      <c r="E72" t="s">
+      <c r="F72" t="s">
         <v>2432</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="30">
         <v>46002</v>
       </c>
       <c r="B73">
         <v>11</v>
       </c>
-      <c r="E73" t="s">
+      <c r="F73" t="s">
         <v>2433</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="30">
         <v>46005</v>
       </c>
@@ -41723,11 +41825,11 @@
       <c r="D74" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E74" s="18" t="s">
+      <c r="F74" s="18" t="s">
         <v>2447</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" s="30">
         <v>46006</v>
       </c>
@@ -41740,11 +41842,11 @@
       <c r="D75" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E75" t="s">
+      <c r="F75" t="s">
         <v>2458</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" s="30">
         <v>46007</v>
       </c>
@@ -41757,11 +41859,11 @@
       <c r="D76" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E76" t="s">
+      <c r="F76" t="s">
         <v>2434</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" s="30">
         <v>46013</v>
       </c>
@@ -41774,11 +41876,11 @@
       <c r="D77" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E77" t="s">
+      <c r="F77" t="s">
         <v>2452</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="30">
         <v>46017</v>
       </c>
@@ -41791,11 +41893,11 @@
       <c r="D78" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E78" t="s">
+      <c r="F78" t="s">
         <v>2439</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" s="30">
         <v>46021</v>
       </c>
@@ -41808,11 +41910,11 @@
       <c r="D79" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E79" t="s">
+      <c r="F79" t="s">
         <v>2448</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" s="30">
         <v>46022</v>
       </c>
@@ -41820,59 +41922,59 @@
         <v>28</v>
       </c>
       <c r="D80" s="57"/>
-      <c r="E80" t="s">
+      <c r="F80" t="s">
         <v>2440</v>
       </c>
-      <c r="I80">
+      <c r="J80">
         <f>(A80-A44)/37</f>
         <v>2.7837837837837838</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="30">
         <v>46028</v>
       </c>
       <c r="B81">
         <v>26</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
         <v>2441</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="30">
         <v>46033</v>
       </c>
       <c r="B82">
         <v>26</v>
       </c>
-      <c r="E82" t="s">
+      <c r="F82" t="s">
         <v>2442</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="30">
         <v>46034</v>
       </c>
       <c r="B83">
         <v>27</v>
       </c>
-      <c r="E83" t="s">
+      <c r="F83" t="s">
         <v>2444</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="30">
         <v>45670</v>
       </c>
       <c r="B84">
         <v>23</v>
       </c>
-      <c r="E84" t="s">
+      <c r="F84" t="s">
         <v>2443</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="30">
         <v>46037</v>
       </c>
@@ -41885,11 +41987,11 @@
       <c r="D85" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E85" t="s">
-        <v>2465</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F85" t="s">
+        <v>2464</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="30">
         <v>46040</v>
       </c>
@@ -41902,11 +42004,11 @@
       <c r="D86" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E86" t="s">
+      <c r="F86" t="s">
         <v>2445</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="30">
         <v>46042</v>
       </c>
@@ -41919,22 +42021,25 @@
       <c r="D87" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E87" t="s">
-        <v>2466</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F87" t="s">
+        <v>2465</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="30">
         <v>46050</v>
       </c>
       <c r="B88">
         <v>27</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E88" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F88" t="s">
         <v>2449</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="30">
         <v>46052</v>
       </c>
@@ -41947,53 +42052,62 @@
       <c r="D89" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E89" t="s">
+      <c r="F89" t="s">
         <v>2450</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90" s="30">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="61">
         <v>46054</v>
       </c>
       <c r="B90">
         <v>24</v>
       </c>
-      <c r="C90" s="50" t="s">
-        <v>2461</v>
+      <c r="C90" s="56" t="s">
+        <v>687</v>
       </c>
       <c r="D90" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E90" s="50" t="s">
+        <v>2476</v>
+      </c>
+      <c r="F90" t="s">
         <v>2451</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A91" s="30">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="62">
         <v>46056</v>
       </c>
       <c r="B91">
         <v>18</v>
       </c>
       <c r="D91" s="57"/>
-      <c r="E91" t="s">
+      <c r="E91" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F91" t="s">
         <v>2453</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A92" s="30">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" s="62">
         <v>46058</v>
       </c>
       <c r="B92">
         <v>26</v>
       </c>
       <c r="D92" s="57"/>
-      <c r="E92" t="s">
+      <c r="E92" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F92" t="s">
         <v>2454</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A93" s="30">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" s="62">
         <v>46059</v>
       </c>
       <c r="B93">
@@ -42005,36 +42119,45 @@
       <c r="D93" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E93" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F93" t="s">
         <v>2455</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A94" s="30">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" s="62">
         <v>46061</v>
       </c>
       <c r="B94">
         <v>20</v>
       </c>
       <c r="D94" s="57"/>
-      <c r="E94" t="s">
+      <c r="E94" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F94" t="s">
         <v>2456</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="30">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" s="62">
         <v>46062</v>
       </c>
       <c r="B95">
         <v>9</v>
       </c>
       <c r="D95" s="57"/>
-      <c r="E95" t="s">
+      <c r="E95" s="50" t="s">
+        <v>2476</v>
+      </c>
+      <c r="F95" t="s">
         <v>2457</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A96" s="30">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" s="62">
         <v>46068</v>
       </c>
       <c r="B96">
@@ -42046,12 +42169,15 @@
       <c r="D96" s="56" t="s">
         <v>2460</v>
       </c>
-      <c r="E96" t="s">
+      <c r="E96" s="50" t="s">
+        <v>2475</v>
+      </c>
+      <c r="F96" t="s">
         <v>2462</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A97" s="30">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97" s="62">
         <v>46075</v>
       </c>
       <c r="B97">
@@ -42063,77 +42189,156 @@
       <c r="D97" s="50" t="s">
         <v>2446</v>
       </c>
-      <c r="E97" t="s">
+      <c r="E97" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F97" t="s">
         <v>2463</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A98" s="30">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A98" s="62">
         <v>46076</v>
       </c>
       <c r="B98">
         <v>18</v>
       </c>
-      <c r="E98" t="s">
-        <v>2464</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A99" s="30">
+      <c r="D98" s="57"/>
+      <c r="E98" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F98" t="s">
+        <v>2478</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A99" s="62">
         <v>46080</v>
       </c>
       <c r="B99">
         <v>20</v>
       </c>
-      <c r="E99" t="s">
-        <v>2467</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A100" s="30">
+      <c r="E99" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F99" t="s">
+        <v>2466</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A100" s="63">
         <v>46086</v>
       </c>
       <c r="B100">
         <v>20</v>
       </c>
-      <c r="E100" t="s">
-        <v>2470</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A101" s="30"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A102" s="30"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A103" s="30"/>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A104" s="30"/>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A105" s="30"/>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A106" s="30"/>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E100" s="50" t="s">
+        <v>2475</v>
+      </c>
+      <c r="F100" t="s">
+        <v>2469</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101" s="64">
+        <v>46089</v>
+      </c>
+      <c r="B101">
+        <v>16</v>
+      </c>
+      <c r="C101" s="50" t="s">
+        <v>2461</v>
+      </c>
+      <c r="D101" s="56" t="s">
+        <v>2460</v>
+      </c>
+      <c r="E101" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F101" t="s">
+        <v>2471</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" s="64">
+        <v>46090</v>
+      </c>
+      <c r="B102">
+        <v>16</v>
+      </c>
+      <c r="C102" s="50" t="s">
+        <v>2461</v>
+      </c>
+      <c r="D102" s="50" t="s">
+        <v>2446</v>
+      </c>
+      <c r="E102" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F102" t="s">
+        <v>2473</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" s="64">
+        <v>46091</v>
+      </c>
+      <c r="B103">
+        <v>16</v>
+      </c>
+      <c r="D103" s="50" t="s">
+        <v>2446</v>
+      </c>
+      <c r="E103" s="50" t="s">
+        <v>2475</v>
+      </c>
+      <c r="F103" t="s">
+        <v>2474</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104" s="64">
+        <v>46093</v>
+      </c>
+      <c r="B104">
+        <v>14</v>
+      </c>
+      <c r="D104" s="50" t="s">
+        <v>2446</v>
+      </c>
+      <c r="E104" s="60" t="s">
+        <v>2472</v>
+      </c>
+      <c r="F104" t="s">
+        <v>2477</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105" s="65" t="s">
+        <v>2479</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A106" s="65" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" s="30"/>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" s="30"/>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" s="30"/>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="30"/>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" s="30"/>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" s="30"/>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Post SSS Commit - not cleaned up
Commit immediately following SSS 'release to org' on 2026-04-14. Includes code for final plots. SCubed2025.py is the main driver program.
</commit_message>
<xml_diff>
--- a/Catalog/Catalog-static.xlsx
+++ b/Catalog/Catalog-static.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Astronomy\Projects\SAS 2021 Ammonia\Jupiter_NH3_Analysis_P3\Catalog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3438C8C6-C23C-4F42-99F4-F8AA3B2F1152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322ADFD4-C105-4D03-B3D5-59501F5552A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5959" uniqueCount="2482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5962" uniqueCount="2485">
   <si>
     <t>ObsID</t>
   </si>
@@ -7903,6 +7903,15 @@
   </si>
   <si>
     <t>Poor to worse focus, Maybe some good NEDFs; 5/25/2025 - processed one observation; Leah's software confused two obskeys, had to manually remove "b" and reletter c-k to b-l</t>
+  </si>
+  <si>
+    <t>Did the last obskey get processed - possible error in V2 s/w 20250324 ??</t>
+  </si>
+  <si>
+    <t>Good seeing, very good transparency.</t>
+  </si>
+  <si>
+    <t>CW</t>
   </si>
 </sst>
 </file>
@@ -8387,7 +8396,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -8502,6 +8511,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -8547,7 +8571,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -8653,6 +8677,18 @@
     <xf numFmtId="0" fontId="0" fillId="50" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="41" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -40753,7 +40789,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99FB822E-4FB0-4362-8846-871BD8F7A1EF}">
-  <dimension ref="A1:J623"/>
+  <dimension ref="A1:J624"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.7265625" customWidth="1"/>
@@ -40769,8 +40805,8 @@
         <v>685</v>
       </c>
       <c r="B1" s="18">
-        <f>SUM(B2:B157)</f>
-        <v>1483</v>
+        <f>SUM(B2:B158)</f>
+        <v>1493</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>695</v>
@@ -41526,8 +41562,11 @@
       <c r="C49" s="56" t="s">
         <v>687</v>
       </c>
-      <c r="D49" s="50" t="s">
-        <v>2445</v>
+      <c r="D49" s="56" t="s">
+        <v>2459</v>
+      </c>
+      <c r="F49" t="s">
+        <v>2482</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
@@ -42036,7 +42075,7 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A88" s="30">
+      <c r="A88" s="61">
         <v>46050</v>
       </c>
       <c r="B88">
@@ -42123,8 +42162,8 @@
       <c r="B93">
         <v>25</v>
       </c>
-      <c r="C93" s="50" t="s">
-        <v>2460</v>
+      <c r="C93" s="56" t="s">
+        <v>687</v>
       </c>
       <c r="D93" s="56" t="s">
         <v>2459</v>
@@ -42351,7 +42390,7 @@
         <v>2480</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="61">
         <v>46101</v>
       </c>
@@ -42365,29 +42404,46 @@
         <v>2480</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A108" s="61"/>
-      <c r="E108" s="60"/>
+    <row r="108" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A108" s="63">
+        <v>46103</v>
+      </c>
+      <c r="B108" s="64">
+        <v>1</v>
+      </c>
+      <c r="C108" s="65"/>
+      <c r="D108" s="65"/>
+      <c r="E108" s="65"/>
+      <c r="F108" s="66" t="s">
+        <v>2484</v>
+      </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A109" s="61"/>
-      <c r="E109" s="60"/>
+      <c r="A109" s="30">
+        <v>46117</v>
+      </c>
+      <c r="B109">
+        <v>9</v>
+      </c>
+      <c r="F109" t="s">
+        <v>2483</v>
+      </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="30"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A111" s="62" t="s">
-        <v>2478</v>
-      </c>
+      <c r="A111" s="30"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" s="62" t="s">
+        <v>2478</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113" s="62" t="s">
         <v>2479</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A113" s="30"/>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A114" s="30"/>
@@ -43918,6 +43974,9 @@
     </row>
     <row r="623" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A623" s="30"/>
+    </row>
+    <row r="624" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A624" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>